<commit_message>
Update stats for 2026-09
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -1227,25 +1227,25 @@
         <v>46266</v>
       </c>
       <c r="B34" t="n">
-        <v>6918</v>
+        <v>6917</v>
       </c>
       <c r="C34" t="n">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="D34" t="n">
-        <v>6991621</v>
+        <v>6989996</v>
       </c>
       <c r="E34" t="n">
-        <v>1010.641948540041</v>
+        <v>1010.55312996964</v>
       </c>
       <c r="F34" t="n">
-        <v>9.757258448357931</v>
+        <v>9.741392987466281</v>
       </c>
       <c r="G34" t="n">
-        <v>8.826479438314937</v>
+        <v>8.625877632898703</v>
       </c>
       <c r="H34" t="n">
-        <v>19.17396984864666</v>
+        <v>19.14627130763533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update stats for 2026-10
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1248,6 +1248,32 @@
         <v>20.05365846590992</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B35" t="n">
+        <v>6930</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1089</v>
+      </c>
+      <c r="D35" t="n">
+        <v>7047753</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1016.991774891775</v>
+      </c>
+      <c r="F35" t="n">
+        <v>9.54789756560228</v>
+      </c>
+      <c r="G35" t="n">
+        <v>8.791208791208781</v>
+      </c>
+      <c r="H35" t="n">
+        <v>18.94239158868252</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>